<commit_message>
feat: add batch run report files in YAML and TXT formats for analysis tracking
</commit_message>
<xml_diff>
--- a/example_project/Analysis/MG_motility/all_brightness.xlsx
+++ b/example_project/Analysis/MG_motility/all_brightness.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,31 +413,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>project tag</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tag folders</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>projection center</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>source image</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>t_i</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Normalized (btw. 0 and 1) average brightness of each stack</t>
         </is>
@@ -468,14 +466,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="n">
-        <v>0.3382042043868631</v>
+      <c r="G2" t="n">
+        <v>0.4789348603784139</v>
       </c>
     </row>
     <row r="3">
@@ -491,14 +499,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
-        <v>0.3412006865559873</v>
+      <c r="G3" t="n">
+        <v>0.4789256686527739</v>
       </c>
     </row>
     <row r="4">
@@ -514,14 +532,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>2</v>
       </c>
-      <c r="E4" t="n">
-        <v>0.3422954267005698</v>
+      <c r="G4" t="n">
+        <v>0.479580056480746</v>
       </c>
     </row>
     <row r="5">
@@ -537,14 +565,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>3</v>
       </c>
-      <c r="E5" t="n">
-        <v>0.3545269193162819</v>
+      <c r="G5" t="n">
+        <v>0.4863881657027835</v>
       </c>
     </row>
     <row r="6">
@@ -560,14 +598,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>4</v>
       </c>
-      <c r="E6" t="n">
-        <v>0.3524090043167931</v>
+      <c r="G6" t="n">
+        <v>0.4840699985939727</v>
       </c>
     </row>
     <row r="7">
@@ -583,14 +631,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>5</v>
       </c>
-      <c r="E7" t="n">
-        <v>0.3526685837934962</v>
+      <c r="G7" t="n">
+        <v>0.4851718476607333</v>
       </c>
     </row>
     <row r="8">
@@ -606,14 +664,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>6</v>
       </c>
-      <c r="E8" t="n">
-        <v>0.3440764213876461</v>
+      <c r="G8" t="n">
+        <v>0.4817485936256083</v>
       </c>
     </row>
     <row r="9">
@@ -629,20 +697,30 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>projection_center_23</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ID240103_P17_1/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>7</v>
       </c>
-      <c r="E9" t="n">
-        <v>0.3443539543254857</v>
+      <c r="G9" t="n">
+        <v>0.4830532405281847</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -652,20 +730,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" t="n">
-        <v>0.4789348603784139</v>
+      <c r="G10" t="n">
+        <v>0.5288621755081883</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -675,20 +763,30 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>1</v>
       </c>
-      <c r="E11" t="n">
-        <v>0.4789256686527739</v>
+      <c r="G11" t="n">
+        <v>0.528961211089791</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -698,20 +796,30 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>2</v>
       </c>
-      <c r="E12" t="n">
-        <v>0.479580056480746</v>
+      <c r="G12" t="n">
+        <v>0.5290850756906206</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -721,20 +829,30 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>3</v>
       </c>
-      <c r="E13" t="n">
-        <v>0.4863881657027835</v>
+      <c r="G13" t="n">
+        <v>0.5294181910508869</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -744,20 +862,30 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
         <v>4</v>
       </c>
-      <c r="E14" t="n">
-        <v>0.4840699985939727</v>
+      <c r="G14" t="n">
+        <v>0.5311076809857636</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -767,20 +895,30 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
         <v>5</v>
       </c>
-      <c r="E15" t="n">
-        <v>0.4851718476607333</v>
+      <c r="G15" t="n">
+        <v>0.5309264791330714</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -790,20 +928,30 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>6</v>
       </c>
-      <c r="E16" t="n">
-        <v>0.4817485936256083</v>
+      <c r="G16" t="n">
+        <v>0.531163293060163</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ID240103_P17_1</t>
+          <t>ID240321_P17_3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -813,197 +961,23 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
+          <t>TP000/registered</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>projection_center_28</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ID240321_P17_3/TP000/registered/all stacks 4D reg.tif</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
         <v>7</v>
       </c>
-      <c r="E17" t="n">
-        <v>0.4830532405281847</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.5288621755081883</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.528961211089791</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.5290850756906206</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.5294181910508869</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>4</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.5311076809857636</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>5</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0.5309264791330714</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>6</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0.531163293060163</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ID240321_P17_3</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>TP000</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>projection_center_28</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>7</v>
-      </c>
-      <c r="E25" t="n">
+      <c r="G17" t="n">
         <v>0.5312566508227039</v>
       </c>
     </row>

</xml_diff>